<commit_message>
Drop extra below_detection column; only fill IL1b_pgml
Leave the workbook structure untouched apart from replacing empty/NA
and <10 values in IL1b_pgml with the 10 pg/mL floor, so the MOI 0
points appear on the log-scale plot.

https://claude.ai/code/session_01DtqFt7Ngb8bywfrWgyFezD
</commit_message>
<xml_diff>
--- a/ELISA_processed.xlsx
+++ b/ELISA_processed.xlsx
@@ -509,11 +509,6 @@
           <t>IL1b_pgml</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>below_detection</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -539,9 +534,6 @@
       <c r="E2" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -567,9 +559,6 @@
       <c r="E3" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F3" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -595,9 +584,6 @@
       <c r="E4" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F4" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -623,9 +609,6 @@
       <c r="E5" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F5" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -651,9 +634,6 @@
       <c r="E6" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F6" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -679,9 +659,6 @@
       <c r="E7" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F7" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -707,9 +684,6 @@
       <c r="E8" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F8" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -735,9 +709,6 @@
       <c r="E9" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F9" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -763,9 +734,6 @@
       <c r="E10" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F10" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -791,9 +759,6 @@
       <c r="E11" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F11" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -819,9 +784,6 @@
       <c r="E12" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F12" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -847,9 +809,6 @@
       <c r="E13" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F13" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -875,9 +834,6 @@
       <c r="E14" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F14" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -903,9 +859,6 @@
       <c r="E15" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F15" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -931,9 +884,6 @@
       <c r="E16" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F16" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -959,9 +909,6 @@
       <c r="E17" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F17" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -987,9 +934,6 @@
       <c r="E18" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F18" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1015,9 +959,6 @@
       <c r="E19" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F19" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1043,9 +984,6 @@
       <c r="E20" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F20" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1071,9 +1009,6 @@
       <c r="E21" s="2" t="n">
         <v>17.49081073</v>
       </c>
-      <c r="F21" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1099,9 +1034,6 @@
       <c r="E22" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F22" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1127,9 +1059,6 @@
       <c r="E23" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F23" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1155,9 +1084,6 @@
       <c r="E24" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F24" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1183,9 +1109,6 @@
       <c r="E25" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F25" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1211,9 +1134,6 @@
       <c r="E26" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F26" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1239,9 +1159,6 @@
       <c r="E27" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F27" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1267,9 +1184,6 @@
       <c r="E28" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F28" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1295,9 +1209,6 @@
       <c r="E29" s="2" t="n">
         <v>31.98182082</v>
       </c>
-      <c r="F29" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1323,9 +1234,6 @@
       <c r="E30" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F30" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1351,9 +1259,6 @@
       <c r="E31" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F31" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1379,9 +1284,6 @@
       <c r="E32" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F32" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1407,9 +1309,6 @@
       <c r="E33" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F33" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1435,9 +1334,6 @@
       <c r="E34" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F34" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1463,9 +1359,6 @@
       <c r="E35" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F35" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1491,9 +1384,6 @@
       <c r="E36" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F36" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1519,9 +1409,6 @@
       <c r="E37" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F37" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1547,9 +1434,6 @@
       <c r="E38" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F38" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1575,9 +1459,6 @@
       <c r="E39" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F39" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1603,9 +1484,6 @@
       <c r="E40" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F40" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1631,9 +1509,6 @@
       <c r="E41" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F41" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1659,9 +1534,6 @@
       <c r="E42" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F42" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1687,9 +1559,6 @@
       <c r="E43" s="2" t="n">
         <v>10.50832956</v>
       </c>
-      <c r="F43" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1715,9 +1584,6 @@
       <c r="E44" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F44" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -1743,9 +1609,6 @@
       <c r="E45" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F45" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -1771,9 +1634,6 @@
       <c r="E46" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F46" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -1799,9 +1659,6 @@
       <c r="E47" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F47" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -1827,9 +1684,6 @@
       <c r="E48" s="2" t="n">
         <v>14.96744341</v>
       </c>
-      <c r="F48" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -1855,9 +1709,6 @@
       <c r="E49" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F49" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -1883,9 +1734,6 @@
       <c r="E50" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F50" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -1911,9 +1759,6 @@
       <c r="E51" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F51" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -1939,9 +1784,6 @@
       <c r="E52" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F52" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -1967,9 +1809,6 @@
       <c r="E53" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F53" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -1995,9 +1834,6 @@
       <c r="E54" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F54" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -2023,9 +1859,6 @@
       <c r="E55" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F55" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -2051,9 +1884,6 @@
       <c r="E56" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F56" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -2079,9 +1909,6 @@
       <c r="E57" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F57" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -2107,9 +1934,6 @@
       <c r="E58" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F58" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -2135,9 +1959,6 @@
       <c r="E59" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F59" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -2163,9 +1984,6 @@
       <c r="E60" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F60" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -2191,9 +2009,6 @@
       <c r="E61" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F61" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -2219,9 +2034,6 @@
       <c r="E62" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F62" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -2247,9 +2059,6 @@
       <c r="E63" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F63" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -2275,9 +2084,6 @@
       <c r="E64" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F64" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -2303,9 +2109,6 @@
       <c r="E65" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F65" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -2331,9 +2134,6 @@
       <c r="E66" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F66" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -2359,9 +2159,6 @@
       <c r="E67" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F67" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -2387,9 +2184,6 @@
       <c r="E68" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F68" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -2415,9 +2209,6 @@
       <c r="E69" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F69" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -2443,9 +2234,6 @@
       <c r="E70" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F70" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -2471,9 +2259,6 @@
       <c r="E71" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F71" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -2499,9 +2284,6 @@
       <c r="E72" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F72" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -2527,9 +2309,6 @@
       <c r="E73" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F73" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -2555,9 +2334,6 @@
       <c r="E74" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F74" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -2583,9 +2359,6 @@
       <c r="E75" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F75" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -2611,9 +2384,6 @@
       <c r="E76" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F76" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -2639,9 +2409,6 @@
       <c r="E77" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F77" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -2667,9 +2434,6 @@
       <c r="E78" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F78" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -2695,9 +2459,6 @@
       <c r="E79" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F79" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -2723,9 +2484,6 @@
       <c r="E80" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F80" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -2751,9 +2509,6 @@
       <c r="E81" s="2" t="n">
         <v>22.19271756</v>
       </c>
-      <c r="F81" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -2779,9 +2534,6 @@
       <c r="E82" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F82" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -2807,9 +2559,6 @@
       <c r="E83" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F83" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -2835,9 +2584,6 @@
       <c r="E84" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F84" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -2863,9 +2609,6 @@
       <c r="E85" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F85" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -2891,9 +2634,6 @@
       <c r="E86" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F86" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -2919,9 +2659,6 @@
       <c r="E87" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F87" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -2947,9 +2684,6 @@
       <c r="E88" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F88" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -2975,9 +2709,6 @@
       <c r="E89" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F89" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -3003,9 +2734,6 @@
       <c r="E90" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F90" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -3031,9 +2759,6 @@
       <c r="E91" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F91" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -3059,9 +2784,6 @@
       <c r="E92" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F92" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -3087,9 +2809,6 @@
       <c r="E93" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F93" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -3115,9 +2834,6 @@
       <c r="E94" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F94" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -3143,9 +2859,6 @@
       <c r="E95" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F95" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -3171,9 +2884,6 @@
       <c r="E96" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F96" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -3199,9 +2909,6 @@
       <c r="E97" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F97" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -3227,9 +2934,6 @@
       <c r="E98" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F98" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -3255,9 +2959,6 @@
       <c r="E99" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F99" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -3283,9 +2984,6 @@
       <c r="E100" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F100" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -3311,9 +3009,6 @@
       <c r="E101" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F101" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -3339,9 +3034,6 @@
       <c r="E102" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F102" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -3367,9 +3059,6 @@
       <c r="E103" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F103" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -3395,9 +3084,6 @@
       <c r="E104" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F104" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -3423,9 +3109,6 @@
       <c r="E105" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F105" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -3451,9 +3134,6 @@
       <c r="E106" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F106" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -3479,9 +3159,6 @@
       <c r="E107" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F107" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -3507,9 +3184,6 @@
       <c r="E108" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F108" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -3535,9 +3209,6 @@
       <c r="E109" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F109" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -3563,9 +3234,6 @@
       <c r="E110" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F110" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -3591,9 +3259,6 @@
       <c r="E111" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F111" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -3619,9 +3284,6 @@
       <c r="E112" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F112" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -3647,9 +3309,6 @@
       <c r="E113" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F113" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -3675,9 +3334,6 @@
       <c r="E114" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F114" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -3703,9 +3359,6 @@
       <c r="E115" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F115" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -3731,9 +3384,6 @@
       <c r="E116" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F116" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -3759,9 +3409,6 @@
       <c r="E117" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F117" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -3787,9 +3434,6 @@
       <c r="E118" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F118" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -3815,9 +3459,6 @@
       <c r="E119" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F119" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -3843,9 +3484,6 @@
       <c r="E120" s="2" t="n">
         <v>86.84910721</v>
       </c>
-      <c r="F120" t="b">
-        <v>0</v>
-      </c>
       <c r="J120" s="3" t="n"/>
     </row>
     <row r="121">
@@ -3872,9 +3510,6 @@
       <c r="E121" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F121" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -3900,9 +3535,6 @@
       <c r="E122" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F122" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -3928,9 +3560,6 @@
       <c r="E123" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F123" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -3956,9 +3585,6 @@
       <c r="E124" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F124" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -3984,9 +3610,6 @@
       <c r="E125" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F125" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -4012,9 +3635,6 @@
       <c r="E126" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F126" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -4040,9 +3660,6 @@
       <c r="E127" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F127" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -4068,9 +3685,6 @@
       <c r="E128" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F128" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -4095,9 +3709,6 @@
       </c>
       <c r="E129" s="2" t="n">
         <v>10</v>
-      </c>
-      <c r="F129" t="b">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Apply 10 pg/mL floor to IL6 and TNFa; generate response plots
Extend the same empty/NA and <10 replacement logic from IL1b to the
IL6 and TNFa sheets, and produce log-scale mean ± 95% CI plots per
mediator and stimulus (BCG, LPS) across carprofen doses.

https://claude.ai/code/session_01DtqFt7Ngb8bywfrWgyFezD
</commit_message>
<xml_diff>
--- a/ELISA_processed.xlsx
+++ b/ELISA_processed.xlsx
@@ -3773,7 +3773,9 @@
           <t>L0</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n"/>
+      <c r="E2" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -3871,7 +3873,9 @@
           <t>L0</t>
         </is>
       </c>
-      <c r="E6" s="2" t="n"/>
+      <c r="E6" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3969,7 +3973,9 @@
           <t>L0</t>
         </is>
       </c>
-      <c r="E10" s="2" t="n"/>
+      <c r="E10" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4067,7 +4073,9 @@
           <t>L0</t>
         </is>
       </c>
-      <c r="E14" s="2" t="n"/>
+      <c r="E14" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4165,7 +4173,9 @@
           <t>B0</t>
         </is>
       </c>
-      <c r="E18" s="2" t="n"/>
+      <c r="E18" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -4188,7 +4198,9 @@
           <t>B1</t>
         </is>
       </c>
-      <c r="E19" s="2" t="n"/>
+      <c r="E19" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -4261,7 +4273,9 @@
           <t>B0</t>
         </is>
       </c>
-      <c r="E22" s="2" t="n"/>
+      <c r="E22" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -4284,7 +4298,9 @@
           <t>B1</t>
         </is>
       </c>
-      <c r="E23" s="2" t="n"/>
+      <c r="E23" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -4357,7 +4373,9 @@
           <t>B0</t>
         </is>
       </c>
-      <c r="E26" s="2" t="n"/>
+      <c r="E26" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -4380,7 +4398,9 @@
           <t>B1</t>
         </is>
       </c>
-      <c r="E27" s="2" t="n"/>
+      <c r="E27" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -4453,7 +4473,9 @@
           <t>B0</t>
         </is>
       </c>
-      <c r="E30" s="2" t="n"/>
+      <c r="E30" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -4476,7 +4498,9 @@
           <t>B1</t>
         </is>
       </c>
-      <c r="E31" s="2" t="n"/>
+      <c r="E31" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -4499,7 +4523,9 @@
           <t>B10</t>
         </is>
       </c>
-      <c r="E32" s="2" t="n"/>
+      <c r="E32" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -4522,7 +4548,9 @@
           <t>B100</t>
         </is>
       </c>
-      <c r="E33" s="2" t="n"/>
+      <c r="E33" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -4545,7 +4573,9 @@
           <t>L0</t>
         </is>
       </c>
-      <c r="E34" s="2" t="n"/>
+      <c r="E34" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -4643,7 +4673,9 @@
           <t>L0</t>
         </is>
       </c>
-      <c r="E38" s="2" t="n"/>
+      <c r="E38" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -4741,7 +4773,9 @@
           <t>L0</t>
         </is>
       </c>
-      <c r="E42" s="2" t="n"/>
+      <c r="E42" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -4839,7 +4873,9 @@
           <t>L0</t>
         </is>
       </c>
-      <c r="E46" s="2" t="n"/>
+      <c r="E46" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -4937,7 +4973,9 @@
           <t>B0</t>
         </is>
       </c>
-      <c r="E50" s="2" t="n"/>
+      <c r="E50" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -4960,7 +4998,9 @@
           <t>B1</t>
         </is>
       </c>
-      <c r="E51" s="2" t="n"/>
+      <c r="E51" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -4983,7 +5023,9 @@
           <t>B10</t>
         </is>
       </c>
-      <c r="E52" s="2" t="n"/>
+      <c r="E52" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -5006,7 +5048,9 @@
           <t>B100</t>
         </is>
       </c>
-      <c r="E53" s="2" t="n"/>
+      <c r="E53" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -5029,7 +5073,9 @@
           <t>B0</t>
         </is>
       </c>
-      <c r="E54" s="2" t="n"/>
+      <c r="E54" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -5052,7 +5098,9 @@
           <t>B1</t>
         </is>
       </c>
-      <c r="E55" s="2" t="n"/>
+      <c r="E55" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -5125,7 +5173,9 @@
           <t>B0</t>
         </is>
       </c>
-      <c r="E58" s="2" t="n"/>
+      <c r="E58" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -5148,7 +5198,9 @@
           <t>B1</t>
         </is>
       </c>
-      <c r="E59" s="2" t="n"/>
+      <c r="E59" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -5171,7 +5223,9 @@
           <t>B10</t>
         </is>
       </c>
-      <c r="E60" s="2" t="n"/>
+      <c r="E60" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -5194,7 +5248,9 @@
           <t>B100</t>
         </is>
       </c>
-      <c r="E61" s="2" t="n"/>
+      <c r="E61" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -5217,7 +5273,9 @@
           <t>B0</t>
         </is>
       </c>
-      <c r="E62" s="2" t="n"/>
+      <c r="E62" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -5240,7 +5298,9 @@
           <t>B1</t>
         </is>
       </c>
-      <c r="E63" s="2" t="n"/>
+      <c r="E63" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -5263,7 +5323,9 @@
           <t>B10</t>
         </is>
       </c>
-      <c r="E64" s="2" t="n"/>
+      <c r="E64" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -5286,7 +5348,9 @@
           <t>B100</t>
         </is>
       </c>
-      <c r="E65" s="2" t="n"/>
+      <c r="E65" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -5309,7 +5373,9 @@
           <t>L0</t>
         </is>
       </c>
-      <c r="E66" s="2" t="n"/>
+      <c r="E66" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -5407,7 +5473,9 @@
           <t>L0</t>
         </is>
       </c>
-      <c r="E70" s="2" t="n"/>
+      <c r="E70" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -5505,7 +5573,9 @@
           <t>L0</t>
         </is>
       </c>
-      <c r="E74" s="2" t="n"/>
+      <c r="E74" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -5603,7 +5673,9 @@
           <t>L0</t>
         </is>
       </c>
-      <c r="E78" s="2" t="n"/>
+      <c r="E78" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -5701,7 +5773,9 @@
           <t>B0</t>
         </is>
       </c>
-      <c r="E82" s="2" t="n"/>
+      <c r="E82" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -5724,7 +5798,9 @@
           <t>B1</t>
         </is>
       </c>
-      <c r="E83" s="2" t="n"/>
+      <c r="E83" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -5747,7 +5823,9 @@
           <t>B10</t>
         </is>
       </c>
-      <c r="E84" s="2" t="n"/>
+      <c r="E84" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -5770,7 +5848,9 @@
           <t>B100</t>
         </is>
       </c>
-      <c r="E85" s="2" t="n"/>
+      <c r="E85" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -5793,7 +5873,9 @@
           <t>B0</t>
         </is>
       </c>
-      <c r="E86" s="2" t="n"/>
+      <c r="E86" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -5816,7 +5898,9 @@
           <t>B1</t>
         </is>
       </c>
-      <c r="E87" s="2" t="n"/>
+      <c r="E87" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -5839,7 +5923,9 @@
           <t>B10</t>
         </is>
       </c>
-      <c r="E88" s="2" t="n"/>
+      <c r="E88" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -5862,7 +5948,9 @@
           <t>B100</t>
         </is>
       </c>
-      <c r="E89" s="2" t="n"/>
+      <c r="E89" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -5885,7 +5973,9 @@
           <t>B0</t>
         </is>
       </c>
-      <c r="E90" s="2" t="n"/>
+      <c r="E90" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -5908,7 +5998,9 @@
           <t>B1</t>
         </is>
       </c>
-      <c r="E91" s="2" t="n"/>
+      <c r="E91" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -5931,7 +6023,9 @@
           <t>B10</t>
         </is>
       </c>
-      <c r="E92" s="2" t="n"/>
+      <c r="E92" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -5954,7 +6048,9 @@
           <t>B100</t>
         </is>
       </c>
-      <c r="E93" s="2" t="n"/>
+      <c r="E93" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -5977,7 +6073,9 @@
           <t>B0</t>
         </is>
       </c>
-      <c r="E94" s="2" t="n"/>
+      <c r="E94" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -6000,7 +6098,9 @@
           <t>B1</t>
         </is>
       </c>
-      <c r="E95" s="2" t="n"/>
+      <c r="E95" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -6023,7 +6123,9 @@
           <t>B10</t>
         </is>
       </c>
-      <c r="E96" s="2" t="n"/>
+      <c r="E96" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -6046,7 +6148,9 @@
           <t>B100</t>
         </is>
       </c>
-      <c r="E97" s="2" t="n"/>
+      <c r="E97" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -6069,7 +6173,9 @@
           <t>L0</t>
         </is>
       </c>
-      <c r="E98" s="2" t="n"/>
+      <c r="E98" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -6167,7 +6273,9 @@
           <t>L0</t>
         </is>
       </c>
-      <c r="E102" s="2" t="n"/>
+      <c r="E102" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -6265,7 +6373,9 @@
           <t>L0</t>
         </is>
       </c>
-      <c r="E106" s="2" t="n"/>
+      <c r="E106" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -6363,7 +6473,9 @@
           <t>L0</t>
         </is>
       </c>
-      <c r="E110" s="2" t="n"/>
+      <c r="E110" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -6461,7 +6573,9 @@
           <t>B0</t>
         </is>
       </c>
-      <c r="E114" s="2" t="n"/>
+      <c r="E114" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -6485,7 +6599,7 @@
         </is>
       </c>
       <c r="E115" s="2" t="n">
-        <v>3.59003586</v>
+        <v>10</v>
       </c>
     </row>
     <row r="116">
@@ -6509,7 +6623,9 @@
           <t>B10</t>
         </is>
       </c>
-      <c r="E116" s="2" t="n"/>
+      <c r="E116" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -6532,7 +6648,9 @@
           <t>B100</t>
         </is>
       </c>
-      <c r="E117" s="2" t="n"/>
+      <c r="E117" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -6555,7 +6673,9 @@
           <t>B0</t>
         </is>
       </c>
-      <c r="E118" s="2" t="n"/>
+      <c r="E118" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -6578,7 +6698,9 @@
           <t>B1</t>
         </is>
       </c>
-      <c r="E119" s="2" t="n"/>
+      <c r="E119" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -6626,7 +6748,9 @@
           <t>B100</t>
         </is>
       </c>
-      <c r="E121" s="2" t="n"/>
+      <c r="E121" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -6649,7 +6773,9 @@
           <t>B0</t>
         </is>
       </c>
-      <c r="E122" s="2" t="n"/>
+      <c r="E122" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -6672,7 +6798,9 @@
           <t>B1</t>
         </is>
       </c>
-      <c r="E123" s="2" t="n"/>
+      <c r="E123" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -6695,7 +6823,9 @@
           <t>B10</t>
         </is>
       </c>
-      <c r="E124" s="2" t="n"/>
+      <c r="E124" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -6718,7 +6848,9 @@
           <t>B100</t>
         </is>
       </c>
-      <c r="E125" s="2" t="n"/>
+      <c r="E125" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -6741,7 +6873,9 @@
           <t>B0</t>
         </is>
       </c>
-      <c r="E126" s="2" t="n"/>
+      <c r="E126" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -6764,7 +6898,9 @@
           <t>B1</t>
         </is>
       </c>
-      <c r="E127" s="2" t="n"/>
+      <c r="E127" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -6787,7 +6923,9 @@
           <t>B10</t>
         </is>
       </c>
-      <c r="E128" s="2" t="n"/>
+      <c r="E128" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -6810,7 +6948,9 @@
           <t>B100</t>
         </is>
       </c>
-      <c r="E129" s="2" t="n"/>
+      <c r="E129" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6874,7 +7014,9 @@
           <t>L0</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n"/>
+      <c r="E2" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -6972,7 +7114,9 @@
           <t>L0</t>
         </is>
       </c>
-      <c r="E6" s="2" t="n"/>
+      <c r="E6" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -7070,7 +7214,9 @@
           <t>L0</t>
         </is>
       </c>
-      <c r="E10" s="2" t="n"/>
+      <c r="E10" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -7169,7 +7315,9 @@
           <t>L0</t>
         </is>
       </c>
-      <c r="E14" s="2" t="n"/>
+      <c r="E14" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -7217,7 +7365,9 @@
           <t>L10</t>
         </is>
       </c>
-      <c r="E16" s="2" t="n"/>
+      <c r="E16" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -7240,7 +7390,9 @@
           <t>L100</t>
         </is>
       </c>
-      <c r="E17" s="2" t="n"/>
+      <c r="E17" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -7263,7 +7415,9 @@
           <t>B0</t>
         </is>
       </c>
-      <c r="E18" s="2" t="n"/>
+      <c r="E18" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -7361,7 +7515,9 @@
           <t>B0</t>
         </is>
       </c>
-      <c r="E22" s="2" t="n"/>
+      <c r="E22" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -7559,7 +7715,9 @@
           <t>B0</t>
         </is>
       </c>
-      <c r="E30" s="2" t="n"/>
+      <c r="E30" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -7757,7 +7915,9 @@
           <t>L0</t>
         </is>
       </c>
-      <c r="E38" s="2" t="n"/>
+      <c r="E38" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -7855,7 +8015,9 @@
           <t>L0</t>
         </is>
       </c>
-      <c r="E42" s="2" t="n"/>
+      <c r="E42" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -7953,7 +8115,9 @@
           <t>L0</t>
         </is>
       </c>
-      <c r="E46" s="2" t="n"/>
+      <c r="E46" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -8051,7 +8215,9 @@
           <t>B0</t>
         </is>
       </c>
-      <c r="E50" s="2" t="n"/>
+      <c r="E50" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -8074,7 +8240,9 @@
           <t>B1</t>
         </is>
       </c>
-      <c r="E51" s="2" t="n"/>
+      <c r="E51" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -8097,7 +8265,9 @@
           <t>B10</t>
         </is>
       </c>
-      <c r="E52" s="2" t="n"/>
+      <c r="E52" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -8120,7 +8290,9 @@
           <t>B100</t>
         </is>
       </c>
-      <c r="E53" s="2" t="n"/>
+      <c r="E53" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -8143,7 +8315,9 @@
           <t>B0</t>
         </is>
       </c>
-      <c r="E54" s="2" t="n"/>
+      <c r="E54" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -8166,7 +8340,9 @@
           <t>B1</t>
         </is>
       </c>
-      <c r="E55" s="2" t="n"/>
+      <c r="E55" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -8189,7 +8365,9 @@
           <t>B10</t>
         </is>
       </c>
-      <c r="E56" s="2" t="n"/>
+      <c r="E56" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -8237,7 +8415,9 @@
           <t>B0</t>
         </is>
       </c>
-      <c r="E58" s="2" t="n"/>
+      <c r="E58" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -8260,7 +8440,9 @@
           <t>B1</t>
         </is>
       </c>
-      <c r="E59" s="2" t="n"/>
+      <c r="E59" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -8283,7 +8465,9 @@
           <t>B10</t>
         </is>
       </c>
-      <c r="E60" s="2" t="n"/>
+      <c r="E60" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -8331,7 +8515,9 @@
           <t>B0</t>
         </is>
       </c>
-      <c r="E62" s="2" t="n"/>
+      <c r="E62" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -8354,7 +8540,9 @@
           <t>B1</t>
         </is>
       </c>
-      <c r="E63" s="2" t="n"/>
+      <c r="E63" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -8377,7 +8565,9 @@
           <t>B10</t>
         </is>
       </c>
-      <c r="E64" s="2" t="n"/>
+      <c r="E64" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -8400,7 +8590,9 @@
           <t>B100</t>
         </is>
       </c>
-      <c r="E65" s="2" t="n"/>
+      <c r="E65" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -8423,7 +8615,9 @@
           <t>L0</t>
         </is>
       </c>
-      <c r="E66" s="2" t="n"/>
+      <c r="E66" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -8521,7 +8715,9 @@
           <t>L0</t>
         </is>
       </c>
-      <c r="E70" s="2" t="n"/>
+      <c r="E70" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -8619,7 +8815,9 @@
           <t>L0</t>
         </is>
       </c>
-      <c r="E74" s="2" t="n"/>
+      <c r="E74" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -8717,7 +8915,9 @@
           <t>L0</t>
         </is>
       </c>
-      <c r="E78" s="2" t="n"/>
+      <c r="E78" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -8815,7 +9015,9 @@
           <t>B0</t>
         </is>
       </c>
-      <c r="E82" s="2" t="n"/>
+      <c r="E82" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -8838,7 +9040,9 @@
           <t>B1</t>
         </is>
       </c>
-      <c r="E83" s="2" t="n"/>
+      <c r="E83" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -8911,7 +9115,9 @@
           <t>B0</t>
         </is>
       </c>
-      <c r="E86" s="2" t="n"/>
+      <c r="E86" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -8934,7 +9140,9 @@
           <t>B1</t>
         </is>
       </c>
-      <c r="E87" s="2" t="n"/>
+      <c r="E87" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -9007,7 +9215,9 @@
           <t>B0</t>
         </is>
       </c>
-      <c r="E90" s="2" t="n"/>
+      <c r="E90" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -9155,7 +9365,9 @@
           <t>B10</t>
         </is>
       </c>
-      <c r="E96" s="2" t="n"/>
+      <c r="E96" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -9204,7 +9416,7 @@
         </is>
       </c>
       <c r="E98" s="2" t="n">
-        <v>5.367657422</v>
+        <v>10</v>
       </c>
     </row>
     <row r="99">
@@ -9304,7 +9516,7 @@
         </is>
       </c>
       <c r="E102" s="2" t="n">
-        <v>6.250814215</v>
+        <v>10</v>
       </c>
     </row>
     <row r="103">
@@ -9404,7 +9616,7 @@
         </is>
       </c>
       <c r="E106" s="2" t="n">
-        <v>5.808884796</v>
+        <v>10</v>
       </c>
     </row>
     <row r="107">
@@ -9504,7 +9716,7 @@
         </is>
       </c>
       <c r="E110" s="2" t="n">
-        <v>7.580526597</v>
+        <v>10</v>
       </c>
     </row>
     <row r="111">
@@ -9603,7 +9815,9 @@
           <t>B0</t>
         </is>
       </c>
-      <c r="E114" s="2" t="n"/>
+      <c r="E114" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -9701,7 +9915,9 @@
           <t>B0</t>
         </is>
       </c>
-      <c r="E118" s="2" t="n"/>
+      <c r="E118" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -9724,7 +9940,9 @@
           <t>B1</t>
         </is>
       </c>
-      <c r="E119" s="2" t="n"/>
+      <c r="E119" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -9823,7 +10041,7 @@
         </is>
       </c>
       <c r="E123" s="2" t="n">
-        <v>8.470042109</v>
+        <v>10</v>
       </c>
     </row>
     <row r="124">
@@ -9947,7 +10165,9 @@
           <t>B10</t>
         </is>
       </c>
-      <c r="E128" s="2" t="n"/>
+      <c r="E128" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -9971,7 +10191,7 @@
         </is>
       </c>
       <c r="E129" s="2" t="n">
-        <v>6.693414928</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>